<commit_message>
Add conversion-focused LP sections for cold traffic trust and clarity.
Delivery breakdown, inside previews, expanded FAQ, honest trust block, and value stack near offer without fake urgency or income claims.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/paletas-de-whatsapp/produto/Calculadora_Precios_Paletas.xlsx
+++ b/paletas-de-whatsapp/produto/Calculadora_Precios_Paletas.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Calculadora" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ejemplo" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lista de compras" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Menú" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Pedidos" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ejemplo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lista de compras" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Menú" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Pedidos" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +43,15 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006B5E57"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -93,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -103,7 +113,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -473,16 +485,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -530,114 +542,129 @@
           <t>Costo usado</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Empaque/unidad</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Otros costos</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n"/>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Fresas</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>500</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>200</v>
+      </c>
       <c r="E4" s="4">
-        <f>IF(D4*C4=0,0,B4/C4*D4)</f>
-        <v/>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G4" s="4" t="n"/>
+        <f>IF(OR(C4=0,D4=0),0,B4/C4*D4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Leche</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>250</v>
+      </c>
       <c r="E5" s="4">
-        <f>IF(D5*C5=0,0,B5/C5*D5)</f>
-        <v/>
-      </c>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="n"/>
+        <f>IF(OR(C5=0,D5=0),0,B5/C5*D5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Crema</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="E6" s="4">
-        <f>IF(D6*C6=0,0,B6/C6*D6)</f>
-        <v/>
-      </c>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="n"/>
+        <f>IF(OR(C6=0,D6=0),0,B6/C6*D6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Azúcar</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>30</v>
+      </c>
       <c r="E7" s="4">
-        <f>IF(D7*C7=0,0,B7/C7*D7)</f>
-        <v/>
-      </c>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="n"/>
+        <f>IF(OR(C7=0,D7=0),0,B7/C7*D7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>6. Usa 'Lista de compras', 'Menú' y 'Pedidos' para organizarte.</t>
+        </is>
+      </c>
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4">
-        <f>IF(D8*C8=0,0,B8/C8*D8)</f>
-        <v/>
-      </c>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n"/>
+      <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4">
-        <f>IF(D9*C9=0,0,B9/C9*D9)</f>
-        <v/>
-      </c>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="n"/>
+        <f>IF(OR(C9=0,D9=0),0,B9/C9*D9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Tip: Sube este archivo a Google Drive → clic derecho → Abrir con Hojas de cálculo.</t>
+        </is>
+      </c>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4">
-        <f>IF(D10*C10=0,0,B10/C10*D10)</f>
-        <v/>
-      </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n"/>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Los números del ejemplo en 'Ejemplo' son ficticios.</t>
+        </is>
+      </c>
       <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4">
-        <f>IF(D11*C11=0,0,B11/C11*D11)</f>
-        <v/>
-      </c>
-      <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -645,11 +672,9 @@
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4">
-        <f>IF(D12*C12=0,0,B12/C12*D12)</f>
-        <v/>
-      </c>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="n"/>
+        <f>IF(OR(C12=0,D12=0),0,B12/C12*D12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -657,78 +682,144 @@
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4">
-        <f>IF(D13*C13=0,0,B13/C13*D13)</f>
-        <v/>
-      </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="n"/>
+        <f>IF(OR(C13=0,D13=0),0,B13/C13*D13)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Cantidad de paletas producidas:</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>8</v>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>— Costos fijos por tanda —</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Costo total:</t>
-        </is>
-      </c>
-      <c r="B16" s="5">
-        <f>SUM(E4:E13)+SUM(F4:F13)+SUM(G4:G13)</f>
-        <v/>
+          <t>Empaque (costo por unidad):</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Costo por paleta:</t>
-        </is>
-      </c>
-      <c r="B17" s="5">
-        <f>IF(B15=0,0,B16/B15)</f>
-        <v/>
+          <t>Palito (costo por unidad):</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Margen deseado %:</t>
+          <t>Otros costos (gas, etiquetas, etc.):</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>40</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Precio sugerido:</t>
-        </is>
-      </c>
-      <c r="B19" s="5">
-        <f>IF(B18&gt;=100,0,B17/(1-B18/100))</f>
-        <v/>
+          <t>Cantidad de paletas producidas:</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>Costo total ingredientes:</t>
+        </is>
+      </c>
+      <c r="B20" s="6">
+        <f>SUM(E4:E13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Costo empaques (unidad × cantidad):</t>
+        </is>
+      </c>
+      <c r="B21" s="6">
+        <f>(B16+B17)*B19+B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Costo total de producción:</t>
+        </is>
+      </c>
+      <c r="B22" s="6">
+        <f>B20+B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Costo por paleta:</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
+        <f>IF(B19=0,0,B22/B19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Margen deseado %:</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Precio sugerido:</t>
+        </is>
+      </c>
+      <c r="B25" s="6">
+        <f>IF(B24&gt;=100,0,B23/(1-B24/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Ganancia estimada por unidad:</t>
         </is>
       </c>
-      <c r="B20" s="5">
-        <f>B19-B17</f>
-        <v/>
+      <c r="B26" s="6">
+        <f>B25-B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Las celdas en verde se calculan solas. Solo edita ingredientes y costos.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A28:E28"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -741,11 +832,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Ejemplo ilustrativo — Paleta de fresa cremosa</t>
         </is>
@@ -759,27 +863,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Ingrediente</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Costo paquete</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Cant. total</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Cant. usada</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>Costo usado</t>
         </is>
@@ -988,7 +1092,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1012,27 +1116,27 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Ingrediente</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Proveedor</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1095,7 +1199,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1112,27 +1216,27 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Sabor</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Costo estimado</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Precio</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -1146,7 +1250,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1173,42 +1277,42 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Teléfono</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Sabor</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>Pagado</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t>Entregado</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>

</xml_diff>